<commit_message>
#13 Client BOM template edited.
</commit_message>
<xml_diff>
--- a/BOM Format/Client.Bom.Template.xlsx
+++ b/BOM Format/Client.Bom.Template.xlsx
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,19 +71,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -112,7 +99,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -127,18 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF03A4CB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -159,15 +140,6 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -186,52 +158,10 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -281,7 +211,24 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -292,12 +239,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -310,88 +253,53 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -681,11 +589,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
@@ -698,123 +606,97 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="23">
+      <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="23">
+      <c r="B4" s="11">
         <f t="shared" ref="B4:B5" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="23">
+      <c r="B5" s="11">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C5" s="26"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="24"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="19"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="20"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>